<commit_message>
Update Philly BYOB Restaurant.xlsx
</commit_message>
<xml_diff>
--- a/philly_yelp_crawler/data/Philly BYOB Restaurant.xlsx
+++ b/philly_yelp_crawler/data/Philly BYOB Restaurant.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slow3\OneDrive\桌面\GitHubProjects\BYOB\philly_yelp_crawler\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AAD88FF-7E03-48FF-927D-556F4F8D1000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50187E9C-4070-4A6F-B910-0FB190C9C8D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{888A9BF0-2D43-4E31-B177-D5314CD5866A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
   <si>
     <t>Name</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -56,117 +56,78 @@
     <t>1415 W Porter St, Philadelphia, PA 19145, United States</t>
   </si>
   <si>
-    <t>+1 215-389-4252</t>
-  </si>
-  <si>
     <t>Bistro La Baia BYOB</t>
   </si>
   <si>
     <t>1700 Lombard St, Philadelphia, PA 19146, United States</t>
   </si>
   <si>
-    <t>+1 267-687-1561</t>
-  </si>
-  <si>
     <t>Kei Sushi</t>
   </si>
   <si>
     <t>1711 South St, Philadelphia, PA 19146, United States</t>
   </si>
   <si>
-    <t>+1 215-309-2925</t>
-  </si>
-  <si>
     <t>Thai Square Restaurant</t>
   </si>
   <si>
     <t>2521 Christian St, Philadelphia, PA 19146, United States</t>
   </si>
   <si>
-    <t>+1 215-454-6683</t>
-  </si>
-  <si>
     <t>Kichi Omakase</t>
   </si>
   <si>
     <t>112 S 12th St, Philadelphia, PA 19107, United States</t>
   </si>
   <si>
-    <t>+1 215-359-6099</t>
-  </si>
-  <si>
     <t>La Sera Italiana BYOB</t>
   </si>
   <si>
     <t>1608 South St, Philadelphia, PA 19146, United States</t>
   </si>
   <si>
-    <t>+1 267-930-7805</t>
-  </si>
-  <si>
     <t>L'Anima</t>
   </si>
   <si>
     <t>1001 S 17th St, Philadelphia, PA 19146, United States</t>
   </si>
   <si>
-    <t>+1 215-595-2500</t>
-  </si>
-  <si>
     <t>Luna BYOB</t>
   </si>
   <si>
     <t>227 S 20th St, Philadelphia, PA 19103, United States</t>
   </si>
   <si>
-    <t>+1 215-693-2220</t>
-  </si>
-  <si>
     <t>Giorgio On Pine</t>
   </si>
   <si>
     <t>1328 Pine St, Philadelphia, PA 19107, United States</t>
   </si>
   <si>
-    <t>+1 215-545-6265</t>
-  </si>
-  <si>
     <t>Giorgio on Pine II</t>
   </si>
   <si>
     <t>1334 Pine St, Philadelphia, PA 19107, United States</t>
   </si>
   <si>
-    <t>+1 215-545-2482</t>
-  </si>
-  <si>
     <t>Trattoria Carina</t>
   </si>
   <si>
     <t>2201 Spruce St, Philadelphia, PA 19103, United States</t>
   </si>
   <si>
-    <t>+1 215-732-5818</t>
-  </si>
-  <si>
     <t>La Viola Bistro</t>
   </si>
   <si>
     <t>253 S 16th St, Philadelphia, PA 19102, United States</t>
   </si>
   <si>
-    <t>+1 215-735-8630</t>
-  </si>
-  <si>
     <t>Melograno</t>
   </si>
   <si>
     <t>2012 Sansom St, Philadelphia, PA 19103, United States</t>
   </si>
   <si>
-    <t>+1 215-875-8116</t>
-  </si>
-  <si>
     <t>ILLATA</t>
   </si>
   <si>
@@ -179,61 +140,256 @@
     <t>231 S 24th St, Philadelphia, PA 19103, United States</t>
   </si>
   <si>
-    <t>+1 215-703-2010</t>
-  </si>
-  <si>
     <t>Nori Sushi</t>
   </si>
   <si>
     <t>1636 South St, Philadelphia, PA 19146, United States</t>
   </si>
   <si>
-    <t>+1 215-735-6668</t>
-  </si>
-  <si>
     <t>Burrata</t>
   </si>
   <si>
     <t>1247 S 13th St, Philadelphia, PA 19147, United States</t>
   </si>
   <si>
-    <t>+1 215-465-2200</t>
-  </si>
-  <si>
     <t>Mercato</t>
   </si>
   <si>
     <t>1216 Spruce St, Philadelphia, PA 19107, United States</t>
   </si>
   <si>
-    <t>+1 215-985-2962</t>
-  </si>
-  <si>
     <t>Sawatdee</t>
   </si>
   <si>
     <t>534 S 15th St, Philadelphia, PA 19146, United States</t>
   </si>
   <si>
-    <t>+1 215-790-1299</t>
-  </si>
-  <si>
     <t>Kinme</t>
   </si>
   <si>
     <t>1117 Locust St, Philadelphia, PA 19107, United States</t>
   </si>
   <si>
-    <t>+1 215-982-1722</t>
-  </si>
-  <si>
     <t>Helm</t>
   </si>
   <si>
     <t>1303 N 5th St, Philadelphia, PA 19122, United States</t>
   </si>
   <si>
-    <t>+1 215-309-2211</t>
+    <t>Stina</t>
+  </si>
+  <si>
+    <t>1705 Snyder Ave, Philadelphia, PA 19145</t>
+  </si>
+  <si>
+    <t>(215) 337-3455</t>
+  </si>
+  <si>
+    <t>KINTO Cozy &amp; Authentic Georgian Restaurant</t>
+  </si>
+  <si>
+    <t>1144 Frankford Ave, Philadelphia, PA 19125</t>
+  </si>
+  <si>
+    <t>(267) 857-9500</t>
+  </si>
+  <si>
+    <t>Nakama Japanese Cuisines &amp; Omakase</t>
+  </si>
+  <si>
+    <t>45 N 13th St, Philadelphia, PA 19107</t>
+  </si>
+  <si>
+    <t>(267) 876-7080</t>
+  </si>
+  <si>
+    <t>A Mano</t>
+  </si>
+  <si>
+    <t>2244 Fairmount Ave, Philadelphia, PA 19130</t>
+  </si>
+  <si>
+    <t>(215) 236-1114</t>
+  </si>
+  <si>
+    <t>El Chingon Philly</t>
+  </si>
+  <si>
+    <t>1524 S 10th St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t>(267) 239-2131</t>
+  </si>
+  <si>
+    <t>Little Fish BYOB</t>
+  </si>
+  <si>
+    <t>746 S 6th St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t>(267) 455-0172</t>
+  </si>
+  <si>
+    <t>Paffuto</t>
+  </si>
+  <si>
+    <t>1009 S 8th St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t>(215) 282-7262</t>
+  </si>
+  <si>
+    <t>Casa Nostra</t>
+  </si>
+  <si>
+    <t>775 S Front St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t>(215) 975-0055</t>
+  </si>
+  <si>
+    <t>Scannicchio's</t>
+  </si>
+  <si>
+    <t>2500 S Broad St, Philadelphia, PA 19145</t>
+  </si>
+  <si>
+    <t>(215) 468-3900</t>
+  </si>
+  <si>
+    <t>Adoro Restaurant</t>
+  </si>
+  <si>
+    <t>769 E Passyunk Ave, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t>(215) 627-1454</t>
+  </si>
+  <si>
+    <t>Mawn</t>
+  </si>
+  <si>
+    <t>764 S 9th St, Philadelphia, PA 19147</t>
+  </si>
+  <si>
+    <t>Rice &amp; Sambal</t>
+  </si>
+  <si>
+    <t>1911 E Passyunk Ave, Philadelphia, PA 19148</t>
+  </si>
+  <si>
+    <t>(215) 279-7052</t>
+  </si>
+  <si>
+    <t>Vic Sushi Bar</t>
+  </si>
+  <si>
+    <t>2035 Sansom St, Philadelphia, PA 19103</t>
+  </si>
+  <si>
+    <t>(215) 564-4339</t>
+  </si>
+  <si>
+    <t>CHAR</t>
+  </si>
+  <si>
+    <t>310 Master St, Philadelphia, PA 19122</t>
+  </si>
+  <si>
+    <t>(215) 964-9874</t>
+  </si>
+  <si>
+    <t>Elma</t>
+  </si>
+  <si>
+    <t>431 E Girard Ave, Philadelphia, PA 19125</t>
+  </si>
+  <si>
+    <t>Pera Turkish Cuisine</t>
+  </si>
+  <si>
+    <t>944 N 2nd St, Philadelphia, PA 19123</t>
+  </si>
+  <si>
+    <t>(215) 660-9471</t>
+  </si>
+  <si>
+    <t>Hikari Sushi</t>
+  </si>
+  <si>
+    <t>1040 N American St #701, Philadelphia, PA 19123</t>
+  </si>
+  <si>
+    <t>(215) 923-2654</t>
+  </si>
+  <si>
+    <t>Vientiane Café</t>
+  </si>
+  <si>
+    <t>4728 Baltimore Ave, Philadelphia, PA 19143</t>
+  </si>
+  <si>
+    <t>(215) 726-1095</t>
+  </si>
+  <si>
+    <t>(215) 703-2010</t>
+  </si>
+  <si>
+    <t>(267) 687-1561</t>
+  </si>
+  <si>
+    <t>(215) 465-2200</t>
+  </si>
+  <si>
+    <t>(215) 545-6265</t>
+  </si>
+  <si>
+    <t>(215) 545-2482</t>
+  </si>
+  <si>
+    <t>(215) 309-2211</t>
+  </si>
+  <si>
+    <t>(215) 309-2925</t>
+  </si>
+  <si>
+    <t>(215) 359-6099</t>
+  </si>
+  <si>
+    <t>(215) 982-1722</t>
+  </si>
+  <si>
+    <t>(267) 930-7805</t>
+  </si>
+  <si>
+    <t>(215) 735-8630</t>
+  </si>
+  <si>
+    <t>(215) 389-4252</t>
+  </si>
+  <si>
+    <t>(215) 595-2500</t>
+  </si>
+  <si>
+    <t>(215) 693-2220</t>
+  </si>
+  <si>
+    <t>(215) 875-8116</t>
+  </si>
+  <si>
+    <t>(215) 985-2962</t>
+  </si>
+  <si>
+    <t>(215) 735-6668</t>
+  </si>
+  <si>
+    <t>(215) 790-1299</t>
+  </si>
+  <si>
+    <t>(215) 454-6683</t>
+  </si>
+  <si>
+    <t>(215) 732-5818</t>
   </si>
 </sst>
 </file>
@@ -628,10 +784,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87E0B387-5980-4442-AEA4-4B4F0537B43A}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="19.33203125" style="1" customWidth="1"/>
     <col min="4" max="16384" width="8.88671875" style="1"/>
@@ -650,233 +806,428 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>72</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>73</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>17</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>21</v>
+        <v>83</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>84</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>27</v>
+        <v>86</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>29</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>32</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>38</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>39</v>
+        <v>91</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>41</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>46</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>49</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>52</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>58</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>61</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="1" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>64</v>
       </c>
+      <c r="C31" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C40">
+    <sortCondition ref="A2:A40"/>
+  </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>